<commit_message>
generated all the reports on 2026-07-19
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -3926,7 +3926,7 @@
     <t>NDNN-description.md</t>
   </si>
   <si>
-    <t>[{"name":"Implementatiemodel Nudging Down Night Noise","resourceReference":"https://data.vlaanderen.be/doc/implementatiemodel/geluidsmeldingen-en-geluidsmetingen/ontwerpstandaard/2026-05-20"}]</t>
+    <t>[{"name":"Implementatiemodel Nudging Down Night Noise","resourceReference":"https://data.vlaanderen.be/doc/implementatiemodel/geluidsmeldingen-en-geluidsmetingen/"}]</t>
   </si>
   <si>
     <t>Charter NDNN</t>
@@ -24872,13 +24872,13 @@
         <v>29</v>
       </c>
       <c r="D259" s="3" t="s">
-        <v>164</v>
+        <v>30</v>
       </c>
       <c r="E259" s="3" t="s">
         <v>31</v>
       </c>
       <c r="F259" s="4">
-        <v>46126</v>
+        <v>46185</v>
       </c>
       <c r="G259" s="3" t="s">
         <v>1303</v>
@@ -24904,10 +24904,16 @@
       <c r="N259" s="4">
         <v>45957</v>
       </c>
-      <c r="O259" s="3"/>
+      <c r="O259" s="4">
+        <v>46185</v>
+      </c>
       <c r="P259" s="3"/>
-      <c r="Q259" s="3"/>
-      <c r="R259" s="3"/>
+      <c r="Q259" s="4">
+        <v>46124</v>
+      </c>
+      <c r="R259" s="4">
+        <v>46185</v>
+      </c>
       <c r="S259" s="3"/>
       <c r="T259" s="3" t="s">
         <v>105</v>
@@ -39430,17 +39436,17 @@
       <c r="K259" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="L259" s="6" t="b">
-        <v>0</v>
+      <c r="L259" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="M259" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="N259" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="O259" s="6" t="b">
-        <v>0</v>
+      <c r="N259" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O259" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="P259" s="6" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
generated all the reports on 2026-08-02
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5870" uniqueCount="1312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5948" uniqueCount="1325">
   <si>
     <t>title</t>
   </si>
@@ -3948,6 +3948,45 @@
   </si>
   <si>
     <t>[{"name":"Overzicht use cases","resourceReference":"https://github.com/Informatievlaanderen/OSLOthema-NDNN/blob/main/usecases.md"}]</t>
+  </si>
+  <si>
+    <t>Implementatiemodel MAGDA - Voertuigregistraties</t>
+  </si>
+  <si>
+    <t>impl-magda-voertuigregistraties-im.md</t>
+  </si>
+  <si>
+    <t>[{"name":"Implementatiemodel MAGDA - Voertuigregistraties","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/magda/voertuigregistratie"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Vocabularium MAGDA-Voertuigregistraties","resourceReference":"https://implementatie.data.vlaanderen.be/ns/voertuigregistratie"},{"name":"Vocabularium Voertuigregistraties","resourceReference":"https://data.vlaanderen.be/ns/voertuigregistratie"},{"name":"Applicatieprofiel OSLO Persoon","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/persoon-basis"},{"name":"Implementatiemodel OSLO Persoon","resourceReference":"https://data.vlaanderen.be/ns/persoon#"},{"name":"Applicatieprofiel OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/organisatie-basis"},{"name":"Implementatiemodel OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/ns/organisatie#"},{"name":"FOAF Vocabulary Specification","resourceReference":"https://xmlns.com/foaf/spec/"},{"name":"SEMIC Core Person Vocabulary","resourceReference":"https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.2/"},{"name":"W3C The Organization Ontology","resourceReference":"https://www.w3.org/TR/vocab-org/"},{"name":"SEMIC Core Public Organisation Vocabulary","resourceReference":"https://semiceu.github.io/CPOV/releases/2.1.2/"},{"name":"SEMIC Core Business Vocabulary","resourceReference":"https://semiceu.github.io/Core-Business-Vocabulary/releases/2.3.0/"}]</t>
+  </si>
+  <si>
+    <t>OSLOthema-trajectcontrole</t>
+  </si>
+  <si>
+    <t>Vocabularium MAGDA - Voertuigregistraties</t>
+  </si>
+  <si>
+    <t>voc-magda-voertuigregistraties-im.md</t>
+  </si>
+  <si>
+    <t>[{"name":"Vocabularium MAGDA - Voertuigregistraties","resourceReference":"https://implementatie.data.vlaanderen.be/ns/magda/voertuigregistratie"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Implementatiemodel MAGDA-Voertuigregistraties","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/magda/voertuigregistratie"},{"name":"Vocabularium Voertuigregistraties","resourceReference":"https://implementatie.data.vlaanderen.be/ns/voertuigregistratie"},{"name":"Applicatieprofiel OSLO Persoon","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/persoon-basis"},{"name":"Vocabularium OSLO Persoon","resourceReference":"https://data.vlaanderen.be/ns/persoon#"},{"name":"Applicatieprofiel OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/organisatie-basis"},{"name":"Vocabularium OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/ns/organisatie#"},{"name":"FOAF Vocabulary Specification","resourceReference":"https://xmlns.com/foaf/spec/"},{"name":"SEMIC Core Person Vocabulary","resourceReference":"https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.2/"},{"name":"W3C The Organization Ontology","resourceReference":"https://www.w3.org/TR/vocab-org/"},{"name":"SEMIC Core Public Organisation Vocabulary","resourceReference":"https://semiceu.github.io/CPOV/releases/2.1.2/"},{"name":"SEMIC Core Business Vocabulary","resourceReference":"https://semiceu.github.io/Core-Business-Vocabulary/releases/2.3.0/"}]</t>
+  </si>
+  <si>
+    <t>Vocabularium Voertuigregistraties</t>
+  </si>
+  <si>
+    <t>voc-voertuigregistraties.md</t>
+  </si>
+  <si>
+    <t>[{"name":"Vocabularium Voertuigregistraties","resourceReference":"https://data.vlaanderen.be/ns/voertuigregistratie"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Implementatiemodel MAGDA-Voertuigregistraties","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/magda/voertuigregistratie"},{"name":"Vocabularium MAGDA-Voertuigregistraties","resourceReference":"https://implementatie.data.vlaanderen.be/ns/magda/voertuigregistratie"},{"name":"Schema.org","resourceReference":"https://schema.org"}]</t>
   </si>
 </sst>
 </file>
@@ -4355,7 +4394,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AA259"/>
+  <dimension ref="A1:AA262"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="27" width="44" customWidth="1"/>
@@ -24937,6 +24976,255 @@
         <v>39</v>
       </c>
       <c r="AA259" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="260" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A260" s="3" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B260" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C260" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D260" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E260" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F260" s="4">
+        <v>46234</v>
+      </c>
+      <c r="G260" s="3" t="s">
+        <v>1313</v>
+      </c>
+      <c r="H260" s="3" t="s">
+        <v>1314</v>
+      </c>
+      <c r="I260" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J260" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K260" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L260" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M260" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N260" s="4">
+        <v>46106</v>
+      </c>
+      <c r="O260" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P260" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q260" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="R260" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S260" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="T260" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="U260" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="V260" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W260" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="X260" s="3" t="s">
+        <v>1315</v>
+      </c>
+      <c r="Y260" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z260" s="3" t="s">
+        <v>1316</v>
+      </c>
+      <c r="AA260" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="261" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A261" s="3" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B261" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C261" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D261" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E261" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F261" s="4">
+        <v>46234</v>
+      </c>
+      <c r="G261" s="3" t="s">
+        <v>1318</v>
+      </c>
+      <c r="H261" s="3" t="s">
+        <v>1319</v>
+      </c>
+      <c r="I261" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J261" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K261" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L261" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M261" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N261" s="4">
+        <v>46106</v>
+      </c>
+      <c r="O261" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P261" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q261" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="R261" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S261" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="T261" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="U261" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="V261" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W261" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="X261" s="3" t="s">
+        <v>1320</v>
+      </c>
+      <c r="Y261" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z261" s="3" t="s">
+        <v>1316</v>
+      </c>
+      <c r="AA261" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="262" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A262" s="3" t="s">
+        <v>1321</v>
+      </c>
+      <c r="B262" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C262" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D262" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E262" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F262" s="4">
+        <v>46234</v>
+      </c>
+      <c r="G262" s="3" t="s">
+        <v>1322</v>
+      </c>
+      <c r="H262" s="3" t="s">
+        <v>1323</v>
+      </c>
+      <c r="I262" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J262" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K262" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L262" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M262" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N262" s="4">
+        <v>46106</v>
+      </c>
+      <c r="O262" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P262" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q262" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="R262" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S262" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="T262" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="U262" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="V262" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W262" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="X262" s="3" t="s">
+        <v>1324</v>
+      </c>
+      <c r="Y262" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z262" s="3" t="s">
+        <v>1316</v>
+      </c>
+      <c r="AA262" s="3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -24948,7 +25236,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R259"/>
+  <dimension ref="A1:R262"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="18" width="44" customWidth="1"/>
@@ -39458,6 +39746,174 @@
         <v>1</v>
       </c>
     </row>
+    <row r="260" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A260" s="3" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G260" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I260" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J260" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O260" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q260" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="R260" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="261" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A261" s="3" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G261" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I261" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J261" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O261" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q261" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="R261" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="262" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A262" s="3" t="s">
+        <v>1321</v>
+      </c>
+      <c r="B262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G262" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I262" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J262" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O262" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q262" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="R262" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
generated all the reports on 2026-08-09
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5948" uniqueCount="1325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6026" uniqueCount="1338">
   <si>
     <t>title</t>
   </si>
@@ -3987,6 +3987,45 @@
   </si>
   <si>
     <t>[{"name":"Implementatiemodel MAGDA-Voertuigregistraties","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/magda/voertuigregistratie"},{"name":"Vocabularium MAGDA-Voertuigregistraties","resourceReference":"https://implementatie.data.vlaanderen.be/ns/magda/voertuigregistratie"},{"name":"Schema.org","resourceReference":"https://schema.org"}]</t>
+  </si>
+  <si>
+    <t>Implementatiemodel Landbouwgebruiksperceel</t>
+  </si>
+  <si>
+    <t>impl-lv-landbouwgebruiksperceel.md</t>
+  </si>
+  <si>
+    <t>[{"name":"Implementatiemodel Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/lv/landbouwgebruiksperceel"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Vocabularium Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/ns/lv/landbouwgebruiksperceel#"},{"name":"Vocabularium Gebruiksperceel","resourceReference":"https://data.vlaanderen.be/ns/gebruiksperceel#"},{"name":"Applicatieprofiel OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/organisatie-basis"},{"name":"Vocabularium OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/ns/organisatie#"},{"name":"Applicatieprofiel OSLO Persoon","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/persoon-basis"},{"name":"Vocabularium OSLO Persoon","resourceReference":"https://data.vlaanderen.be/ns/persoon#"},{"name":"W3C The Organization Ontology","resourceReference":"https://www.w3.org/TR/vocab-org/"},{"name":"SEMIC Core Public Organisation Vocabulary","resourceReference":"https://semiceu.github.io/CPOV/releases/2.1.2/"},{"name":"SEMIC Core Business Vocabulary","resourceReference":"https://semiceu.github.io/Core-Business-Vocabulary/releases/2.3.0/"},{"name":"SEMIC Core Person Vocabulary","resourceReference":"https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.2/"}]</t>
+  </si>
+  <si>
+    <t>OSLOthema-landbouwgebruiksperceel</t>
+  </si>
+  <si>
+    <t>Vocabularium Landbouwgebruiksperceel</t>
+  </si>
+  <si>
+    <t>voc-lv-landbouwgebruiksperceel.md</t>
+  </si>
+  <si>
+    <t>[{"name":"Vocabularium Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/ns/lv/landbouwgebruiksperceel#"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Implementatiemodel Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/lv/landbouwgebruiksperceel"},{"name":"Vocabularium Gebruiksperceel","resourceReference":"https://data.vlaanderen.be/ns/gebruiksperceel#"},{"name":"Applicatieprofiel OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/organisatie-basis"},{"name":"Vocabularium OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/ns/organisatie#"},{"name":"Applicatieprofiel OSLO Persoon","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/persoon-basis"},{"name":"Vocabularium OSLO Persoon","resourceReference":"https://data.vlaanderen.be/ns/persoon#"},{"name":"W3C The Organization Ontology","resourceReference":"https://www.w3.org/TR/vocab-org/"},{"name":"SEMIC Core Public Organisation Vocabulary","resourceReference":"https://semiceu.github.io/CPOV/releases/2.1.2/"},{"name":"SEMIC Core Business Vocabulary","resourceReference":"https://semiceu.github.io/Core-Business-Vocabulary/releases/2.3.0/"},{"name":"SEMIC Core Person Vocabulary","resourceReference":"https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.2/"}]</t>
+  </si>
+  <si>
+    <t>Vocabularium Gebruiksperceel</t>
+  </si>
+  <si>
+    <t>voc-gebruiksperceel.md</t>
+  </si>
+  <si>
+    <t>[{"name":"Vocabularium Gebruiksperceel","resourceReference":"https://data.vlaanderen.be/ns/gebruiksperceel#"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Implementatiemodel Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/lv/landbouwgebruiksperceel"},{"name":"Vocabularium Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/ns/lv/landbouwgebruiksperceel#"}]</t>
   </si>
 </sst>
 </file>
@@ -4394,7 +4433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AA262"/>
+  <dimension ref="A1:AA265"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="27" width="44" customWidth="1"/>
@@ -25225,6 +25264,255 @@
         <v>1316</v>
       </c>
       <c r="AA262" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="263" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A263" s="3" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B263" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C263" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D263" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E263" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F263" s="4">
+        <v>46237</v>
+      </c>
+      <c r="G263" s="3" t="s">
+        <v>1326</v>
+      </c>
+      <c r="H263" s="3" t="s">
+        <v>1327</v>
+      </c>
+      <c r="I263" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J263" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K263" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L263" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M263" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N263" s="4">
+        <v>46175</v>
+      </c>
+      <c r="O263" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P263" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q263" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="R263" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S263" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="T263" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="U263" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="V263" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W263" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="X263" s="3" t="s">
+        <v>1328</v>
+      </c>
+      <c r="Y263" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z263" s="3" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AA263" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="264" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A264" s="3" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D264" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E264" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F264" s="4">
+        <v>46237</v>
+      </c>
+      <c r="G264" s="3" t="s">
+        <v>1331</v>
+      </c>
+      <c r="H264" s="3" t="s">
+        <v>1332</v>
+      </c>
+      <c r="I264" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J264" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K264" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L264" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M264" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N264" s="4">
+        <v>46175</v>
+      </c>
+      <c r="O264" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P264" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q264" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="R264" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S264" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="T264" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="U264" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="V264" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W264" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="X264" s="3" t="s">
+        <v>1333</v>
+      </c>
+      <c r="Y264" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z264" s="3" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AA264" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="265" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A265" s="3" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B265" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C265" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D265" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E265" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F265" s="4">
+        <v>46237</v>
+      </c>
+      <c r="G265" s="3" t="s">
+        <v>1335</v>
+      </c>
+      <c r="H265" s="3" t="s">
+        <v>1336</v>
+      </c>
+      <c r="I265" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J265" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K265" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L265" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M265" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N265" s="4">
+        <v>46175</v>
+      </c>
+      <c r="O265" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P265" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q265" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="R265" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S265" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="T265" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="U265" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="V265" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W265" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="X265" s="3" t="s">
+        <v>1337</v>
+      </c>
+      <c r="Y265" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z265" s="3" t="s">
+        <v>1329</v>
+      </c>
+      <c r="AA265" s="3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -25236,7 +25524,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R262"/>
+  <dimension ref="A1:R265"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="18" width="44" customWidth="1"/>
@@ -39914,6 +40202,174 @@
         <v>1</v>
       </c>
     </row>
+    <row r="263" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A263" s="3" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G263" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I263" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J263" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O263" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q263" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="R263" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="264" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A264" s="3" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G264" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I264" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J264" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O264" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q264" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="R264" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="265" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A265" s="3" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G265" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I265" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J265" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O265" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q265" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="R265" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
generated all the reports on 2026-09-06
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6026" uniqueCount="1338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6005" uniqueCount="1328">
   <si>
     <t>title</t>
   </si>
@@ -3890,36 +3890,6 @@
     <t>Vocabularium Rooilijnplannen</t>
   </si>
   <si>
-    <t>SSN SOSA VL</t>
-  </si>
-  <si>
-    <t>https://data.vlaanderen.be/id/concept/StandaardType/Interoperabiliteit</t>
-  </si>
-  <si>
-    <t>SSNSOSA-description.md</t>
-  </si>
-  <si>
-    <t>[{"name":"Datavoorbeelden SSN SOSA VL","resourceReference":"https://github.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/tree/main/resources"}]</t>
-  </si>
-  <si>
-    <t>Charter SSNSOSAVL</t>
-  </si>
-  <si>
-    <t>https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/charter/Charter_OSLO_SSN%20SOSA%20VL.docx</t>
-  </si>
-  <si>
-    <t>[{"name":"Verslag Business Werkgroep - 3 december 2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/reports/Verslag%20-%20Business%20werkgroep%20SSN%20SOSA%20VL.pdf"},{"name":"Verslag Thematische Werkgroep 1 - 14 januari 2026","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/reports/Verslag%20Thematische%20werkgroep%201%20-%20SSN%20SOSA%20%202026-02-02.pdf"},{"name":"Verslag Thematische Werkgroep 2 - 3 april 2026","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/reports/Verslag%20Thematische%20werkgroep%202%20-%20SSN%20SOSA%20%202026-03-04.pdf"},{"name":"Verslag Thematische Werkgroep 3 - 29 april 2026","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/reports/Verslag%20Thematische%20werkgroep%203%20-%20SSN%20SOSA%20%202026-29-04.pdf"}]</t>
-  </si>
-  <si>
-    <t>[{"name":"Presentatie Business Werkgroep -  3 december 2025","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/presentations/SSN%20SOSA%20VL%20Business%20Werkgroep.pdf"},{"name":"Presentatie Thematische Werkgroep 1 - 14 januari 2026","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/presentations/Presentatie%20SSN%20SOSA%20VL%20Thematische%20werkgroep%201.pdf"},{"name":"Presentatie Thematische Werkgroep 2 - 3 april 2026","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/presentations/Presentatie%20SSN%20SOSA%20VL%20Thematische%20werkgroep%202.pdf"},{"name":"Presentatie Thematische Werkgroep 3 - 29 april 2026","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/presentations/Presentatie%20SSN%20SOSA%20VL%20Thematische%20werkgroep%203.pdf"}]</t>
-  </si>
-  <si>
-    <t>https://data.vlaanderen.be/doc/concept/Domein/Omgeving</t>
-  </si>
-  <si>
-    <t>{"name":"Charter SSNSOSAVL","resourceReference":"https://raw.githubusercontent.com/Informatievlaanderen/OSLOthema-SSNSOSA-VL/standaardenregister/charter/Charter_OSLO_SSN%20SOSA%20VL.docx"}</t>
-  </si>
-  <si>
     <t>Implementatiemodel Geluidsmeldingen en -metingen</t>
   </si>
   <si>
@@ -3998,7 +3968,7 @@
     <t>[{"name":"Implementatiemodel Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/lv/landbouwgebruiksperceel"}]</t>
   </si>
   <si>
-    <t>[{"name":"Vocabularium Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/ns/lv/landbouwgebruiksperceel#"},{"name":"Vocabularium Gebruiksperceel","resourceReference":"https://data.vlaanderen.be/ns/gebruiksperceel#"},{"name":"Applicatieprofiel OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/organisatie-basis"},{"name":"Vocabularium OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/ns/organisatie#"},{"name":"Applicatieprofiel OSLO Persoon","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/persoon-basis"},{"name":"Vocabularium OSLO Persoon","resourceReference":"https://data.vlaanderen.be/ns/persoon#"},{"name":"W3C The Organization Ontology","resourceReference":"https://www.w3.org/TR/vocab-org/"},{"name":"SEMIC Core Public Organisation Vocabulary","resourceReference":"https://semiceu.github.io/CPOV/releases/2.1.2/"},{"name":"SEMIC Core Business Vocabulary","resourceReference":"https://semiceu.github.io/Core-Business-Vocabulary/releases/2.3.0/"},{"name":"SEMIC Core Person Vocabulary","resourceReference":"https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.2/"}]</t>
+    <t>[{"name":"Vocabularium Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/ns/lv/landbouwgebruiksperceel"},{"name":"Vocabularium Gebruiksperceel","resourceReference":"https://data.vlaanderen.be/ns/gebruiksperceel"},{"name":"Applicatieprofiel OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/organisatie-basis"},{"name":"Vocabularium OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/ns/organisatie"},{"name":"Applicatieprofiel OSLO Persoon","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/persoon-basis"},{"name":"Vocabularium OSLO Persoon","resourceReference":"https://data.vlaanderen.be/ns/persoon"},{"name":"W3C The Organization Ontology","resourceReference":"https://www.w3.org/TR/vocab-org/"},{"name":"SEMIC Core Public Organisation Vocabulary","resourceReference":"https://semiceu.github.io/CPOV/releases/2.1.2/"},{"name":"SEMIC Core Business Vocabulary","resourceReference":"https://semiceu.github.io/Core-Business-Vocabulary/releases/2.3.0/"},{"name":"SEMIC Core Person Vocabulary","resourceReference":"https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.2/"}]</t>
   </si>
   <si>
     <t>OSLOthema-landbouwgebruiksperceel</t>
@@ -4010,10 +3980,10 @@
     <t>voc-lv-landbouwgebruiksperceel.md</t>
   </si>
   <si>
-    <t>[{"name":"Vocabularium Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/ns/lv/landbouwgebruiksperceel#"}]</t>
-  </si>
-  <si>
-    <t>[{"name":"Implementatiemodel Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/lv/landbouwgebruiksperceel"},{"name":"Vocabularium Gebruiksperceel","resourceReference":"https://data.vlaanderen.be/ns/gebruiksperceel#"},{"name":"Applicatieprofiel OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/organisatie-basis"},{"name":"Vocabularium OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/ns/organisatie#"},{"name":"Applicatieprofiel OSLO Persoon","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/persoon-basis"},{"name":"Vocabularium OSLO Persoon","resourceReference":"https://data.vlaanderen.be/ns/persoon#"},{"name":"W3C The Organization Ontology","resourceReference":"https://www.w3.org/TR/vocab-org/"},{"name":"SEMIC Core Public Organisation Vocabulary","resourceReference":"https://semiceu.github.io/CPOV/releases/2.1.2/"},{"name":"SEMIC Core Business Vocabulary","resourceReference":"https://semiceu.github.io/Core-Business-Vocabulary/releases/2.3.0/"},{"name":"SEMIC Core Person Vocabulary","resourceReference":"https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.2/"}]</t>
+    <t>[{"name":"Vocabularium Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/ns/lv/landbouwgebruiksperceel"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Implementatiemodel Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/lv/landbouwgebruiksperceel"},{"name":"Vocabularium Gebruiksperceel","resourceReference":"https://data.vlaanderen.be/ns/gebruiksperceel"},{"name":"Applicatieprofiel OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/organisatie-basis"},{"name":"Vocabularium OSLO Organisatie","resourceReference":"https://data.vlaanderen.be/ns/organisatie"},{"name":"Applicatieprofiel OSLO Persoon","resourceReference":"https://data.vlaanderen.be/doc/applicatieprofiel/persoon-basis"},{"name":"Vocabularium OSLO Persoon","resourceReference":"https://data.vlaanderen.be/ns/persoon"},{"name":"W3C The Organization Ontology","resourceReference":"https://www.w3.org/TR/vocab-org/"},{"name":"SEMIC Core Public Organisation Vocabulary","resourceReference":"https://semiceu.github.io/CPOV/releases/2.1.2/"},{"name":"SEMIC Core Business Vocabulary","resourceReference":"https://semiceu.github.io/Core-Business-Vocabulary/releases/2.3.0/"},{"name":"SEMIC Core Person Vocabulary","resourceReference":"https://semiceu.github.io/Core-Person-Vocabulary/releases/2.1.2/"}]</t>
   </si>
   <si>
     <t>Vocabularium Gebruiksperceel</t>
@@ -4022,10 +3992,10 @@
     <t>voc-gebruiksperceel.md</t>
   </si>
   <si>
-    <t>[{"name":"Vocabularium Gebruiksperceel","resourceReference":"https://data.vlaanderen.be/ns/gebruiksperceel#"}]</t>
-  </si>
-  <si>
-    <t>[{"name":"Implementatiemodel Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/lv/landbouwgebruiksperceel"},{"name":"Vocabularium Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/ns/lv/landbouwgebruiksperceel#"}]</t>
+    <t>[{"name":"Vocabularium Gebruiksperceel","resourceReference":"https://data.vlaanderen.be/ns/gebruiksperceel"}]</t>
+  </si>
+  <si>
+    <t>[{"name":"Implementatiemodel Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/doc/implementatiemodel/lv/landbouwgebruiksperceel"},{"name":"Vocabularium Landbouwgebruiksperceel","resourceReference":"https://implementatie.data.vlaanderen.be/ns/lv/landbouwgebruiksperceel"}]</t>
   </si>
 </sst>
 </file>
@@ -4433,7 +4403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AA265"/>
+  <dimension ref="A1:AA264"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="27" width="44" customWidth="1"/>
@@ -24871,51 +24841,57 @@
         <v>1292</v>
       </c>
       <c r="B258" s="3" t="s">
-        <v>1293</v>
+        <v>87</v>
       </c>
       <c r="C258" s="3" t="s">
         <v>29</v>
       </c>
       <c r="D258" s="3" t="s">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="E258" s="3" t="s">
         <v>31</v>
       </c>
       <c r="F258" s="4">
-        <v>46072</v>
+        <v>46185</v>
       </c>
       <c r="G258" s="3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="H258" s="3" t="s">
         <v>1294</v>
       </c>
-      <c r="H258" s="3" t="s">
+      <c r="I258" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I258" s="3" t="s">
+      <c r="J258" s="3" t="s">
         <v>1295</v>
       </c>
-      <c r="J258" s="3" t="s">
+      <c r="K258" s="3" t="s">
         <v>1296</v>
       </c>
-      <c r="K258" s="3" t="s">
+      <c r="L258" s="3" t="s">
         <v>1297</v>
       </c>
-      <c r="L258" s="3" t="s">
+      <c r="M258" s="3" t="s">
         <v>1298</v>
       </c>
-      <c r="M258" s="3" t="s">
-        <v>1299</v>
-      </c>
       <c r="N258" s="4">
-        <v>45974</v>
-      </c>
-      <c r="O258" s="3"/>
+        <v>45957</v>
+      </c>
+      <c r="O258" s="4">
+        <v>46185</v>
+      </c>
       <c r="P258" s="3"/>
-      <c r="Q258" s="3"/>
-      <c r="R258" s="3"/>
+      <c r="Q258" s="4">
+        <v>46124</v>
+      </c>
+      <c r="R258" s="4">
+        <v>46185</v>
+      </c>
       <c r="S258" s="3"/>
       <c r="T258" s="3" t="s">
-        <v>1300</v>
+        <v>105</v>
       </c>
       <c r="U258" s="3" t="s">
         <v>34</v>
@@ -24924,13 +24900,13 @@
         <v>39</v>
       </c>
       <c r="W258" s="3" t="s">
+        <v>1299</v>
+      </c>
+      <c r="X258" s="3" t="s">
+        <v>1300</v>
+      </c>
+      <c r="Y258" s="3" t="s">
         <v>1301</v>
-      </c>
-      <c r="X258" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y258" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="Z258" s="3" t="s">
         <v>39</v>
@@ -24950,13 +24926,13 @@
         <v>29</v>
       </c>
       <c r="D259" s="3" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="E259" s="3" t="s">
         <v>31</v>
       </c>
       <c r="F259" s="4">
-        <v>46185</v>
+        <v>46234</v>
       </c>
       <c r="G259" s="3" t="s">
         <v>1303</v>
@@ -24968,33 +24944,37 @@
         <v>34</v>
       </c>
       <c r="J259" s="3" t="s">
-        <v>1305</v>
+        <v>39</v>
       </c>
       <c r="K259" s="3" t="s">
-        <v>1306</v>
+        <v>39</v>
       </c>
       <c r="L259" s="3" t="s">
-        <v>1307</v>
+        <v>34</v>
       </c>
       <c r="M259" s="3" t="s">
-        <v>1308</v>
+        <v>34</v>
       </c>
       <c r="N259" s="4">
-        <v>45957</v>
-      </c>
-      <c r="O259" s="4">
-        <v>46185</v>
-      </c>
-      <c r="P259" s="3"/>
-      <c r="Q259" s="4">
-        <v>46124</v>
-      </c>
-      <c r="R259" s="4">
-        <v>46185</v>
-      </c>
-      <c r="S259" s="3"/>
+        <v>46106</v>
+      </c>
+      <c r="O259" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P259" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q259" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="R259" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S259" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="T259" s="3" t="s">
-        <v>105</v>
+        <v>126</v>
       </c>
       <c r="U259" s="3" t="s">
         <v>34</v>
@@ -25003,16 +24983,16 @@
         <v>39</v>
       </c>
       <c r="W259" s="3" t="s">
-        <v>1309</v>
+        <v>83</v>
       </c>
       <c r="X259" s="3" t="s">
-        <v>1310</v>
+        <v>1305</v>
       </c>
       <c r="Y259" s="3" t="s">
-        <v>1311</v>
+        <v>34</v>
       </c>
       <c r="Z259" s="3" t="s">
-        <v>39</v>
+        <v>1306</v>
       </c>
       <c r="AA259" s="3" t="s">
         <v>39</v>
@@ -25020,10 +25000,10 @@
     </row>
     <row r="260" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A260" s="3" t="s">
-        <v>1312</v>
+        <v>1307</v>
       </c>
       <c r="B260" s="3" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="C260" s="3" t="s">
         <v>29</v>
@@ -25038,10 +25018,10 @@
         <v>46234</v>
       </c>
       <c r="G260" s="3" t="s">
-        <v>1313</v>
+        <v>1308</v>
       </c>
       <c r="H260" s="3" t="s">
-        <v>1314</v>
+        <v>1309</v>
       </c>
       <c r="I260" s="3" t="s">
         <v>34</v>
@@ -25089,13 +25069,13 @@
         <v>83</v>
       </c>
       <c r="X260" s="3" t="s">
-        <v>1315</v>
+        <v>1310</v>
       </c>
       <c r="Y260" s="3" t="s">
         <v>34</v>
       </c>
       <c r="Z260" s="3" t="s">
-        <v>1316</v>
+        <v>1306</v>
       </c>
       <c r="AA260" s="3" t="s">
         <v>39</v>
@@ -25103,7 +25083,7 @@
     </row>
     <row r="261" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A261" s="3" t="s">
-        <v>1317</v>
+        <v>1311</v>
       </c>
       <c r="B261" s="3" t="s">
         <v>76</v>
@@ -25112,7 +25092,7 @@
         <v>29</v>
       </c>
       <c r="D261" s="3" t="s">
-        <v>77</v>
+        <v>164</v>
       </c>
       <c r="E261" s="3" t="s">
         <v>31</v>
@@ -25121,10 +25101,10 @@
         <v>46234</v>
       </c>
       <c r="G261" s="3" t="s">
-        <v>1318</v>
+        <v>1312</v>
       </c>
       <c r="H261" s="3" t="s">
-        <v>1319</v>
+        <v>1313</v>
       </c>
       <c r="I261" s="3" t="s">
         <v>34</v>
@@ -25172,13 +25152,13 @@
         <v>83</v>
       </c>
       <c r="X261" s="3" t="s">
-        <v>1320</v>
+        <v>1314</v>
       </c>
       <c r="Y261" s="3" t="s">
         <v>34</v>
       </c>
       <c r="Z261" s="3" t="s">
-        <v>1316</v>
+        <v>1306</v>
       </c>
       <c r="AA261" s="3" t="s">
         <v>39</v>
@@ -25186,28 +25166,28 @@
     </row>
     <row r="262" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A262" s="3" t="s">
-        <v>1321</v>
+        <v>1315</v>
       </c>
       <c r="B262" s="3" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="C262" s="3" t="s">
         <v>29</v>
       </c>
       <c r="D262" s="3" t="s">
-        <v>164</v>
+        <v>77</v>
       </c>
       <c r="E262" s="3" t="s">
         <v>31</v>
       </c>
       <c r="F262" s="4">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="G262" s="3" t="s">
-        <v>1322</v>
+        <v>1316</v>
       </c>
       <c r="H262" s="3" t="s">
-        <v>1323</v>
+        <v>1317</v>
       </c>
       <c r="I262" s="3" t="s">
         <v>34</v>
@@ -25225,7 +25205,7 @@
         <v>34</v>
       </c>
       <c r="N262" s="4">
-        <v>46106</v>
+        <v>46175</v>
       </c>
       <c r="O262" s="3" t="s">
         <v>80</v>
@@ -25243,7 +25223,7 @@
         <v>80</v>
       </c>
       <c r="T262" s="3" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="U262" s="3" t="s">
         <v>34</v>
@@ -25255,13 +25235,13 @@
         <v>83</v>
       </c>
       <c r="X262" s="3" t="s">
-        <v>1324</v>
+        <v>1318</v>
       </c>
       <c r="Y262" s="3" t="s">
         <v>34</v>
       </c>
       <c r="Z262" s="3" t="s">
-        <v>1316</v>
+        <v>1319</v>
       </c>
       <c r="AA262" s="3" t="s">
         <v>39</v>
@@ -25269,10 +25249,10 @@
     </row>
     <row r="263" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A263" s="3" t="s">
-        <v>1325</v>
+        <v>1320</v>
       </c>
       <c r="B263" s="3" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="C263" s="3" t="s">
         <v>29</v>
@@ -25287,10 +25267,10 @@
         <v>46237</v>
       </c>
       <c r="G263" s="3" t="s">
-        <v>1326</v>
+        <v>1321</v>
       </c>
       <c r="H263" s="3" t="s">
-        <v>1327</v>
+        <v>1322</v>
       </c>
       <c r="I263" s="3" t="s">
         <v>34</v>
@@ -25338,13 +25318,13 @@
         <v>83</v>
       </c>
       <c r="X263" s="3" t="s">
-        <v>1328</v>
+        <v>1323</v>
       </c>
       <c r="Y263" s="3" t="s">
         <v>34</v>
       </c>
       <c r="Z263" s="3" t="s">
-        <v>1329</v>
+        <v>1319</v>
       </c>
       <c r="AA263" s="3" t="s">
         <v>39</v>
@@ -25352,7 +25332,7 @@
     </row>
     <row r="264" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A264" s="3" t="s">
-        <v>1330</v>
+        <v>1324</v>
       </c>
       <c r="B264" s="3" t="s">
         <v>76</v>
@@ -25361,7 +25341,7 @@
         <v>29</v>
       </c>
       <c r="D264" s="3" t="s">
-        <v>77</v>
+        <v>164</v>
       </c>
       <c r="E264" s="3" t="s">
         <v>31</v>
@@ -25370,10 +25350,10 @@
         <v>46237</v>
       </c>
       <c r="G264" s="3" t="s">
-        <v>1331</v>
+        <v>1325</v>
       </c>
       <c r="H264" s="3" t="s">
-        <v>1332</v>
+        <v>1326</v>
       </c>
       <c r="I264" s="3" t="s">
         <v>34</v>
@@ -25421,98 +25401,15 @@
         <v>83</v>
       </c>
       <c r="X264" s="3" t="s">
-        <v>1333</v>
+        <v>1327</v>
       </c>
       <c r="Y264" s="3" t="s">
         <v>34</v>
       </c>
       <c r="Z264" s="3" t="s">
-        <v>1329</v>
+        <v>1319</v>
       </c>
       <c r="AA264" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="265" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A265" s="3" t="s">
-        <v>1334</v>
-      </c>
-      <c r="B265" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C265" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D265" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="E265" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F265" s="4">
-        <v>46237</v>
-      </c>
-      <c r="G265" s="3" t="s">
-        <v>1335</v>
-      </c>
-      <c r="H265" s="3" t="s">
-        <v>1336</v>
-      </c>
-      <c r="I265" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J265" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="K265" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="L265" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M265" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="N265" s="4">
-        <v>46175</v>
-      </c>
-      <c r="O265" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="P265" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="Q265" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="R265" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="S265" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="T265" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="U265" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="V265" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="W265" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="X265" s="3" t="s">
-        <v>1337</v>
-      </c>
-      <c r="Y265" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z265" s="3" t="s">
-        <v>1329</v>
-      </c>
-      <c r="AA265" s="3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -25524,7 +25421,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R265"/>
+  <dimension ref="A1:R264"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="18" width="44" customWidth="1"/>
@@ -39938,11 +39835,11 @@
       <c r="E258" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="F258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G258" s="5" t="b">
-        <v>1</v>
+      <c r="F258" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G258" s="6" t="b">
+        <v>0</v>
       </c>
       <c r="H258" s="5" t="b">
         <v>1</v>
@@ -39956,17 +39853,17 @@
       <c r="K258" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="L258" s="6" t="b">
-        <v>0</v>
+      <c r="L258" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="M258" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="N258" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="O258" s="6" t="b">
-        <v>0</v>
+      <c r="N258" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O258" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="P258" s="6" t="b">
         <v>0</v>
@@ -40003,11 +39900,11 @@
       <c r="H259" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="I259" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="J259" s="5" t="b">
-        <v>1</v>
+      <c r="I259" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="J259" s="6" t="b">
+        <v>0</v>
       </c>
       <c r="K259" s="5" t="b">
         <v>1</v>
@@ -40015,17 +39912,17 @@
       <c r="L259" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="M259" s="6" t="b">
-        <v>0</v>
+      <c r="M259" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="N259" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="O259" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="P259" s="6" t="b">
-        <v>0</v>
+      <c r="O259" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P259" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="Q259" s="5" t="b">
         <v>1</v>
@@ -40036,7 +39933,7 @@
     </row>
     <row r="260" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A260" s="3" t="s">
-        <v>1312</v>
+        <v>1307</v>
       </c>
       <c r="B260" s="5" t="b">
         <v>1</v>
@@ -40092,7 +39989,7 @@
     </row>
     <row r="261" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A261" s="3" t="s">
-        <v>1317</v>
+        <v>1311</v>
       </c>
       <c r="B261" s="5" t="b">
         <v>1</v>
@@ -40148,7 +40045,7 @@
     </row>
     <row r="262" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A262" s="3" t="s">
-        <v>1321</v>
+        <v>1315</v>
       </c>
       <c r="B262" s="5" t="b">
         <v>1</v>
@@ -40204,7 +40101,7 @@
     </row>
     <row r="263" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A263" s="3" t="s">
-        <v>1325</v>
+        <v>1320</v>
       </c>
       <c r="B263" s="5" t="b">
         <v>1</v>
@@ -40260,7 +40157,7 @@
     </row>
     <row r="264" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A264" s="3" t="s">
-        <v>1330</v>
+        <v>1324</v>
       </c>
       <c r="B264" s="5" t="b">
         <v>1</v>
@@ -40311,62 +40208,6 @@
         <v>1</v>
       </c>
       <c r="R264" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="265" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A265" s="3" t="s">
-        <v>1334</v>
-      </c>
-      <c r="B265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="C265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="D265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G265" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I265" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="J265" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="K265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="L265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="M265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="N265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="O265" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="P265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q265" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="R265" s="5" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
generated all the reports on 2026-09-20
</commit_message>
<xml_diff>
--- a/report/merged_configurations.xlsx
+++ b/report/merged_configurations.xlsx
@@ -24932,7 +24932,7 @@
         <v>31</v>
       </c>
       <c r="F259" s="4">
-        <v>46234</v>
+        <v>46279</v>
       </c>
       <c r="G259" s="3" t="s">
         <v>1303</v>
@@ -25015,7 +25015,7 @@
         <v>31</v>
       </c>
       <c r="F260" s="4">
-        <v>46234</v>
+        <v>46279</v>
       </c>
       <c r="G260" s="3" t="s">
         <v>1308</v>
@@ -25098,7 +25098,7 @@
         <v>31</v>
       </c>
       <c r="F261" s="4">
-        <v>46234</v>
+        <v>46279</v>
       </c>
       <c r="G261" s="3" t="s">
         <v>1312</v>

</xml_diff>